<commit_message>
MOD. Exporta correctamente la version calendario que necesita Pati
</commit_message>
<xml_diff>
--- a/inputs/programacion_matriz.xlsx
+++ b/inputs/programacion_matriz.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\git\Trabajos\programacion_academica\outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\git\Trabajos\programacion_academica\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BF06B4-E5D6-406F-9D6D-9FF5C105A79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8A63D8-714C-47F6-869C-2F342E3ACCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -357,22 +357,26 @@
       <b/>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1630,9 +1634,7 @@
       <c r="D7" s="12"/>
       <c r="E7" s="13"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="13">
-        <v>4</v>
-      </c>
+      <c r="G7" s="13"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
       <c r="J7" s="12">
@@ -1693,7 +1695,9 @@
       </c>
       <c r="AR7" s="12"/>
       <c r="AS7" s="12"/>
-      <c r="AT7" s="12"/>
+      <c r="AT7" s="12">
+        <v>4</v>
+      </c>
       <c r="AU7" s="13"/>
       <c r="AV7" s="13"/>
       <c r="AW7" s="13"/>
@@ -2396,9 +2400,7 @@
       </c>
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
-      <c r="N14" s="15">
-        <v>1.5</v>
-      </c>
+      <c r="N14" s="15"/>
       <c r="O14" s="15"/>
       <c r="P14" s="15"/>
       <c r="Q14" s="13">
@@ -2429,9 +2431,7 @@
       </c>
       <c r="AG14" s="12"/>
       <c r="AH14" s="12"/>
-      <c r="AI14" s="15">
-        <v>1.5</v>
-      </c>
+      <c r="AI14" s="15"/>
       <c r="AJ14" s="15"/>
       <c r="AK14" s="15"/>
       <c r="AL14" s="12">
@@ -2444,37 +2444,43 @@
       </c>
       <c r="AP14" s="13"/>
       <c r="AQ14" s="13"/>
-      <c r="AR14" s="12">
-        <v>1.5</v>
-      </c>
+      <c r="AR14" s="12"/>
       <c r="AS14" s="12"/>
       <c r="AT14" s="12"/>
-      <c r="AU14" s="13"/>
+      <c r="AU14" s="13">
+        <v>1.5</v>
+      </c>
       <c r="AV14" s="13"/>
       <c r="AW14" s="13"/>
-      <c r="AX14" s="12"/>
+      <c r="AX14" s="12">
+        <v>1.5</v>
+      </c>
       <c r="AY14" s="12"/>
       <c r="AZ14" s="12"/>
-      <c r="BA14" s="13"/>
+      <c r="BA14" s="13">
+        <v>1.5</v>
+      </c>
       <c r="BB14" s="13"/>
       <c r="BC14" s="13"/>
-      <c r="BD14" s="12"/>
+      <c r="BD14" s="12">
+        <v>1.5</v>
+      </c>
       <c r="BE14" s="12"/>
       <c r="BF14" s="12"/>
       <c r="BG14" s="16">
         <f t="shared" si="0"/>
-        <v>19.5</v>
+        <v>21</v>
       </c>
       <c r="BH14" s="16">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="BI14" s="16">
         <f t="shared" si="1"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="BJ14" s="18" t="str">
         <f t="shared" si="2"/>
-        <v>Incompleta</v>
+        <v>Completa</v>
       </c>
     </row>
     <row r="16" spans="1:62" x14ac:dyDescent="0.25">
@@ -2497,7 +2503,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="19">
         <f t="shared" ref="G16:V16" si="3">MAX(G5:G6)+MAX(G11:G13)+G7+G8+G9+G10+G14</f>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H16" s="2">
         <f t="shared" si="3"/>
@@ -2525,7 +2531,7 @@
       </c>
       <c r="N16" s="4">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="O16" s="19">
         <f t="shared" si="3"/>
@@ -2600,91 +2606,91 @@
       </c>
       <c r="AI16" s="4">
         <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="19">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="AK16" s="19">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="AL16" s="2">
+        <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="AJ16" s="19">
+      <c r="AM16" s="19">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="AK16" s="19">
+      <c r="AN16" s="19">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="AL16" s="2">
+      <c r="AO16" s="1">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="AM16" s="19">
+      <c r="AP16" s="19">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="AN16" s="19">
+      <c r="AQ16" s="19">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="AO16" s="1">
+      <c r="AR16" s="2">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AS16" s="19">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="AT16" s="19">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="AU16" s="1">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="AP16" s="19">
+      <c r="AV16" s="19">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="AQ16" s="19">
-        <f t="shared" si="4"/>
-        <v>10</v>
-      </c>
-      <c r="AR16" s="2">
+      <c r="AW16" s="19">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="AX16" s="2">
         <f t="shared" si="4"/>
         <v>1.5</v>
       </c>
-      <c r="AS16" s="19">
+      <c r="AY16" s="19">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="AT16" s="19">
+      <c r="AZ16" s="19">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="AU16" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AV16" s="19">
+      <c r="BA16" s="1">
+        <f t="shared" si="4"/>
+        <v>1.5</v>
+      </c>
+      <c r="BB16" s="19">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="AW16" s="19">
+      <c r="BC16" s="19">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="AX16" s="2">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AY16" s="19">
-        <f t="shared" si="4"/>
-        <v>7</v>
-      </c>
-      <c r="AZ16" s="19">
-        <f t="shared" si="4"/>
-        <v>6</v>
-      </c>
-      <c r="BA16" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="BB16" s="19">
-        <f t="shared" si="4"/>
-        <v>7</v>
-      </c>
-      <c r="BC16" s="19">
-        <f t="shared" si="4"/>
-        <v>6</v>
-      </c>
       <c r="BD16" s="2">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="BE16" s="19">
         <f t="shared" si="4"/>

</xml_diff>